<commit_message>
feat(F-NAR-019): TREE-COL-009 polish Le bouton rouge de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-009.xlsx
+++ b/stories/arbres/TREE-COL-009.xlsx
@@ -5239,17 +5239,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Nina range le bouton dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable se ferme sur la virgule de fil.</t>
+          <t>Nina range le bouton dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable garde la plume et la perle, au chaud.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina range le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable se ferme sur la virgule de fil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina range le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable garde la plume et la perle, au chaud.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina range le &lt;emphasis&gt;bouton&lt;/emphasis&gt; dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable se ferme sur la virgule de fil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina range le &lt;emphasis&gt;bouton&lt;/emphasis&gt; dans le cartable. Une plume et une perle de yaourt voyagent ensemble. Ils se touchent, dans la poche. On le coud à la maison ? Oui, le fil est long. Le cube bosselé rentre aussi ? Oui, près du rouge. Le cartable garde la plume et la perle, au chaud.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5394,7 +5394,7 @@
 enfant-f|Oui, le fil est long.
 maman|Le cube bosselé rentre aussi ?
 enfant-f|Oui, près du rouge.
-narrateur|Le cartable se ferme sur la virgule de fil.</t>
+narrateur|Le cartable garde la plume et la perle, au chaud.</t>
         </is>
       </c>
       <c r="AX23" t="inlineStr">
@@ -15942,17 +15942,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Nina range bouton et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. Le cartable se ferme sur la virgule de fil.</t>
+          <t>Nina range bouton et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. La tasse cliquette une fois, puis plus rien.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina range &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. Le cartable se ferme sur la virgule de fil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina range &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. La tasse cliquette une fois, puis plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina range &lt;emphasis&gt;bouton&lt;/emphasis&gt; et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. Le cartable se ferme sur la virgule de fil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina range &lt;emphasis&gt;bouton&lt;/emphasis&gt; et tasse dans le cartable. Une plume colle à la perle de yaourt. La cerise voyage. On coud ce soir ? Oui, le fil est long. La dînette rentre aussi ? La tasse, oui. La tasse cliquette une fois, puis plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -16097,7 +16097,7 @@
 enfant-f|Oui, le fil est long.
 maman|La dînette rentre aussi ?
 enfant-f|La tasse, oui.
-narrateur|Le cartable se ferme sur la virgule de fil.</t>
+narrateur|La tasse cliquette une fois, puis plus rien.</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
@@ -16714,17 +16714,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. Le manteau ferme, le crochet reste vide.</t>
+          <t>Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. La casserole de dînette reste tiède, vide.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. Le manteau ferme, le crochet reste vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. La casserole de dînette reste tiède, vide.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. Le manteau ferme, le crochet reste vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina recoud au coin du crochet, la casserole à côté. Une miette et un poil de chat partagent le fil. Le trou est juste ? Juste. La dînette sent le pain, un peu. Le tic du radiateur suit le dernier point. La casserole de dînette reste tiède, vide.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16868,7 +16868,7 @@
 enfant-f|Juste.
 maman|La dînette sent le pain, un peu.
 narrateur|Le tic du radiateur suit le dernier point.
-narrateur|Le manteau ferme, le crochet reste vide.</t>
+narrateur|La casserole de dînette reste tiède, vide.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17469,17 +17469,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Nina glisse le bouton dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. La virgule de fil dépasse, comme un secret.</t>
+          <t>Nina glisse le bouton dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. Une plume pique le col, tout léger.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina glisse le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. La virgule de fil dépasse, comme un secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina glisse le &lt;emphasis level="moderate"&gt;bouton&lt;/emphasis&gt; dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. Une plume pique le col, tout léger.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina glisse le &lt;emphasis&gt;bouton&lt;/emphasis&gt; dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. La virgule de fil dépasse, comme un secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina glisse le &lt;emphasis&gt;bouton&lt;/emphasis&gt; dans le manteau, dehors. Une plume et une miette tiennent au fil. Ça raconte la poule, et le gâteau. La dînette rentre ? Oui, la soupe pour de rire est finie. Le trou est plein, maintenant ? Plein. Une plume pique le col, tout léger.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17624,7 +17624,7 @@
 enfant-f|Oui, la soupe pour de rire est finie.
 maman|Le trou est plein, maintenant ?
 enfant-f|Plein.
-narrateur|La virgule de fil dépasse, comme un secret.</t>
+narrateur|Une plume pique le col, tout léger.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
@@ -17650,7 +17650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17707,6 +17707,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>